<commit_message>
Usun duplikat pyt. 61 z pliku 2016 i popraw liraglutyd w ARCYBAZIE
- pyt. 61 (Glikokortykosteroidy zmniejszaja liczbe) bylo dokladnym duplikatem
  pyt. 61 z egzaminu 2014/2015 - usuniete z pliku 2016 (99 -> 98 pytan),
  odnotowane w slowniku POMINIETE z podana przyczyna
- liraglutyd oznaczony jako poprawna odpowiedz w pytaniu Terapia cukrzycy
  typu 2 podskornie (agonista GLP-1 podawany podskornie, potwierdzone przez
  uzytkowniczke); zapisane w CORRECTIONS, przetrwa regeneracje pliku

Kontrola: 0 duplikatow w calym zestawie, 0 wierszy wadliwych, 0 trafien
detektora zanieczyszczen, importer 1084/1239.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017sDWkA2eXfHxFn4vQGjL1J
</commit_message>
<xml_diff>
--- a/farmakologia_egzamin_2016_OnlyPharms.xlsx
+++ b/farmakologia_egzamin_2016_OnlyPharms.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Pytania" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pytania'!$A$1:$O$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pytania'!$A$1:$O$99</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O100"/>
+  <dimension ref="A1:O99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -3625,7 +3625,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>GLIKOKORTYKOSTEROIDY</t>
+          <t>CUKRZYCA</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -3641,32 +3641,32 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>Glikokortykosteroidy zmniejszają liczbę:</t>
+          <t>Wskaż właściwe stwierdzenia odnoszące się do pramlintydu:</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>monocytów</t>
+          <t>redukuje glikemię poposiłkową</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>limfocytów</t>
-        </is>
-      </c>
-      <c r="H61" s="2" t="inlineStr"/>
+          <t>hamuje sekrecję glukagonu</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr">
+        <is>
+          <t>zwalnia opróżnianie żołądka</t>
+        </is>
+      </c>
       <c r="I61" s="2" t="inlineStr"/>
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="2" t="inlineStr">
         <is>
-          <t>płytek krwi</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr">
-        <is>
-          <t>neutrofili</t>
-        </is>
-      </c>
+          <t>zwiększa apetyt</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr"/>
       <c r="N61" s="2" t="inlineStr"/>
       <c r="O61" s="2" t="inlineStr"/>
@@ -3674,7 +3674,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>CUKRZYCA</t>
+          <t>FARMAKOKINETYKA</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -3690,33 +3690,33 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Wskaż właściwe stwierdzenia odnoszące się do pramlintydu:</t>
+          <t>Inhibitor allosteryczny:</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>redukuje glikemię poposiłkową</t>
-        </is>
-      </c>
-      <c r="G62" s="2" t="inlineStr">
-        <is>
-          <t>hamuje sekrecję glukagonu</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>zwalnia opróżnianie żołądka</t>
-        </is>
-      </c>
+          <t>zmniejsza odpowiedź po związaniu się agonisty z receptorem</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr">
         <is>
-          <t>zwiększa apetyt</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="inlineStr"/>
-      <c r="M62" s="2" t="inlineStr"/>
+          <t>uniemożliwia połączenie się agonisty z receptorem</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>zmienia strukturę III-rzędową agonisty</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>wiąże się z agonistą i neutralizuje jego działanie</t>
+        </is>
+      </c>
       <c r="N62" s="2" t="inlineStr"/>
       <c r="O62" s="2" t="inlineStr"/>
     </row>
@@ -3728,7 +3728,7 @@
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>Mechanizm działania</t>
+          <t>Farmakokinetyka</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr"/>
@@ -3739,33 +3739,33 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>Inhibitor allosteryczny:</t>
+          <t>Leki prekursorowe są aktywowane do postaci aktywnych:</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>zmniejsza odpowiedź po związaniu się agonisty z receptorem</t>
-        </is>
-      </c>
-      <c r="G63" s="2" t="inlineStr"/>
-      <c r="H63" s="2" t="inlineStr"/>
+          <t>w wątrobie</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>w osoczu</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr">
+        <is>
+          <t>w nabłonku jelita</t>
+        </is>
+      </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>uniemożliwia połączenie się agonisty z receptorem</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>zmienia strukturę III-rzędową agonisty</t>
-        </is>
-      </c>
-      <c r="M63" s="2" t="inlineStr">
-        <is>
-          <t>wiąże się z agonistą i neutralizuje jego działanie</t>
-        </is>
-      </c>
+          <t>w śledzionie</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr"/>
+      <c r="M63" s="2" t="inlineStr"/>
       <c r="N63" s="2" t="inlineStr"/>
       <c r="O63" s="2" t="inlineStr"/>
     </row>
@@ -3788,29 +3788,29 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Leki prekursorowe są aktywowane do postaci aktywnych:</t>
+          <t>Duża objętość dystrybucji leku może sugerować:</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>w wątrobie</t>
+          <t>istnienie kompartmentu głębokiego, czyli narządu kumulującego lek</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr">
         <is>
-          <t>w osoczu</t>
+          <t>małą szybkość wydalania</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>w nabłonku jelita</t>
+          <t>dużą lipofilność</t>
         </is>
       </c>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="inlineStr"/>
       <c r="K64" s="2" t="inlineStr">
         <is>
-          <t>w śledzionie</t>
+          <t>dużą zawartość wody w organizmie</t>
         </is>
       </c>
       <c r="L64" s="2" t="inlineStr"/>
@@ -3821,12 +3821,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>FARMAKOKINETYKA</t>
+          <t>LEKI PRZECIWDEPRESYJNE</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Farmakokinetyka</t>
+          <t>Działania niepożądane</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr"/>
@@ -3837,45 +3837,57 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Duża objętość dystrybucji leku może sugerować:</t>
+          <t>Węglan litu powoduje:</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>istnienie kompartmentu głębokiego, czyli narządu kumulującego lek</t>
+          <t>drżenie</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>małą szybkość wydalania</t>
+          <t>zaburzenia czynności tarczycy</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>dużą lipofilność</t>
-        </is>
-      </c>
-      <c r="I65" s="2" t="inlineStr"/>
+          <t>polidypsję</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>obrzęki</t>
+        </is>
+      </c>
       <c r="J65" s="2" t="inlineStr"/>
       <c r="K65" s="2" t="inlineStr">
         <is>
-          <t>dużą zawartość wody w organizmie</t>
-        </is>
-      </c>
-      <c r="L65" s="2" t="inlineStr"/>
-      <c r="M65" s="2" t="inlineStr"/>
+          <t>agranulocytozę</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>zwłóknienie płuc</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>methemoglobinemię</t>
+        </is>
+      </c>
       <c r="N65" s="2" t="inlineStr"/>
       <c r="O65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>LEKI PRZECIWDEPRESYJNE</t>
+          <t>HEMOSTAZA</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Działania niepożądane</t>
+          <t>Mechanizm działania</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr"/>
@@ -3886,45 +3898,33 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Węglan litu powoduje:</t>
+          <t>Wskaż właściwe stwierdzenia odnoszące się do prasugrelu:</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>drżenie</t>
+          <t>jest prolekiem</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>zaburzenia czynności tarczycy</t>
+          <t>wiąże się trwale z receptorem P2Y12 na płytkach krwi</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
-          <t>polidypsję</t>
-        </is>
-      </c>
-      <c r="I66" s="2" t="inlineStr">
-        <is>
-          <t>obrzęki</t>
-        </is>
-      </c>
+          <t>może być podawany łącznie z kwasem acetylosalicylowym</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="2" t="inlineStr">
         <is>
-          <t>agranulocytozę</t>
-        </is>
-      </c>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>zwłóknienie płuc</t>
-        </is>
-      </c>
-      <c r="M66" s="2" t="inlineStr">
-        <is>
-          <t>methemoglobinemię</t>
-        </is>
-      </c>
+          <t>jest podawany w profilaktyce migotania przedsionków u pacjentów z przeciwwskazaniem do stosowania antagonistów witaminy K</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="2" t="inlineStr"/>
       <c r="N66" s="2" t="inlineStr"/>
       <c r="O66" s="2" t="inlineStr"/>
     </row>
@@ -3947,29 +3947,29 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Wskaż właściwe stwierdzenia odnoszące się do prasugrelu:</t>
+          <t>Wskaż właściwe stwierdzenia odnoszące się do eteksylanu dabigatranu:</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>jest prolekiem</t>
+          <t>swoiście i odwracalnie hamuje trombinę</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>wiąże się trwale z receptorem P2Y12 na płytkach krwi</t>
+          <t>jest lekiem prekursorowym</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
-          <t>może być podawany łącznie z kwasem acetylosalicylowym</t>
+          <t>jest skuteczny w zapobieganiu powikłaniom zakrzepowym migotania przedsionków</t>
         </is>
       </c>
       <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="2" t="inlineStr"/>
       <c r="K67" s="2" t="inlineStr">
         <is>
-          <t>jest podawany w profilaktyce migotania przedsionków u pacjentów z przeciwwskazaniem do stosowania antagonistów witaminy K</t>
+          <t>podczas stosowania wymaga monitorowania układu krzepnięcia</t>
         </is>
       </c>
       <c r="L67" s="2" t="inlineStr"/>
@@ -3980,12 +3980,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>HEMOSTAZA</t>
+          <t>LEKI PRZECIWBAKTERYJNE</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>Mechanizm działania</t>
+          <t>Sposób podania</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr"/>
@@ -3996,29 +3996,29 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Wskaż właściwe stwierdzenia odnoszące się do eteksylanu dabigatranu:</t>
+          <t>Wskaż właściwe stwierdzenia odnoszące się do chlorheksydyny:</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>swoiście i odwracalnie hamuje trombinę</t>
+          <t>stosowana jest w wodnych preparatach w postaci diglukonianu chlorheksydyny</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>jest lekiem prekursorowym</t>
+          <t>ma niewielkie działanie uczulające lub drażniące skórę</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
-          <t>jest skuteczny w zapobieganiu powikłaniom zakrzepowym migotania przedsionków</t>
+          <t>jest przeciwwskazana podczas operacji w uchu środkowym</t>
         </is>
       </c>
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" s="2" t="inlineStr">
         <is>
-          <t>podczas stosowania wymaga monitorowania układu krzepnięcia</t>
+          <t>jest odporna na działanie środków powierzchniowo czynnych</t>
         </is>
       </c>
       <c r="L68" s="2" t="inlineStr"/>
@@ -4034,7 +4034,7 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>Sposób podania</t>
+          <t>Interakcje</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr"/>
@@ -4045,32 +4045,32 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Wskaż właściwe stwierdzenia odnoszące się do chlorheksydyny:</t>
+          <t>Reakcję disulfiramową może wywołać:</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>stosowana jest w wodnych preparatach w postaci diglukonianu chlorheksydyny</t>
+          <t>cefamandol</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>ma niewielkie działanie uczulające lub drażniące skórę</t>
-        </is>
-      </c>
-      <c r="H69" s="2" t="inlineStr">
-        <is>
-          <t>jest przeciwwskazana podczas operacji w uchu środkowym</t>
-        </is>
-      </c>
+          <t>metronidazol</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr"/>
       <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="2" t="inlineStr"/>
       <c r="K69" s="2" t="inlineStr">
         <is>
-          <t>jest odporna na działanie środków powierzchniowo czynnych</t>
-        </is>
-      </c>
-      <c r="L69" s="2" t="inlineStr"/>
+          <t>oksazepam</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>metformina</t>
+        </is>
+      </c>
       <c r="M69" s="2" t="inlineStr"/>
       <c r="N69" s="2" t="inlineStr"/>
       <c r="O69" s="2" t="inlineStr"/>
@@ -4078,12 +4078,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>LEKI PRZECIWBAKTERYJNE</t>
+          <t>CHOROBA PARKINSONA</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>Interakcje</t>
+          <t>Działania niepożądane</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr"/>
@@ -4094,40 +4094,44 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Reakcję disulfiramową może wywołać:</t>
+          <t>Wady zastawek serca mogą wystąpić podczas leczenia:</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>cefamandol</t>
-        </is>
-      </c>
-      <c r="G70" s="2" t="inlineStr">
-        <is>
-          <t>metronidazol</t>
-        </is>
-      </c>
+          <t>pergolid</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr"/>
       <c r="H70" s="2" t="inlineStr"/>
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr">
         <is>
-          <t>oksazepam</t>
+          <t>selegilina</t>
         </is>
       </c>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>metformina</t>
-        </is>
-      </c>
-      <c r="M70" s="2" t="inlineStr"/>
-      <c r="N70" s="2" t="inlineStr"/>
+          <t>entakapon</t>
+        </is>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>amantadyna</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>procyklidyna</t>
+        </is>
+      </c>
       <c r="O70" s="2" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>CHOROBA PARKINSONA</t>
+          <t>PADACZKA</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -4143,12 +4147,12 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>Wady zastawek serca mogą wystąpić podczas leczenia:</t>
+          <t>Ubytki w polu widzenia mogą wystąpić podczas leczenia:</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
-          <t>pergolid</t>
+          <t>wigabatryna</t>
         </is>
       </c>
       <c r="G71" s="2" t="inlineStr"/>
@@ -4157,22 +4161,22 @@
       <c r="J71" s="2" t="inlineStr"/>
       <c r="K71" s="2" t="inlineStr">
         <is>
-          <t>selegilina</t>
+          <t>zonisamid</t>
         </is>
       </c>
       <c r="L71" s="2" t="inlineStr">
         <is>
-          <t>entakapon</t>
+          <t>gabapentyna</t>
         </is>
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>amantadyna</t>
+          <t>pregabalina</t>
         </is>
       </c>
       <c r="N71" s="2" t="inlineStr">
         <is>
-          <t>procyklidyna</t>
+          <t>lamotrygina</t>
         </is>
       </c>
       <c r="O71" s="2" t="inlineStr"/>
@@ -4180,12 +4184,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>PADACZKA</t>
+          <t>UKŁAD ODDECHOWY</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Działania niepożądane</t>
+          <t>Mechanizm działania</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr"/>
@@ -4196,12 +4200,12 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Ubytki w polu widzenia mogą wystąpić podczas leczenia:</t>
+          <t>Omalizumab:</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>wigabatryna</t>
+          <t>jest przeciwciałem monoklonalnym anty-IgE</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr"/>
@@ -4210,22 +4214,22 @@
       <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr">
         <is>
-          <t>zonisamid</t>
+          <t>hamuje fosfodiesterazę typu 2</t>
         </is>
       </c>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>gabapentyna</t>
+          <t>jest agonistą receptorów beta-2</t>
         </is>
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>pregabalina</t>
+          <t>hamuje fosfolipazę A2</t>
         </is>
       </c>
       <c r="N72" s="2" t="inlineStr">
         <is>
-          <t>lamotrygina</t>
+          <t>działa hamująco na receptory dla leukotrienów</t>
         </is>
       </c>
       <c r="O72" s="2" t="inlineStr"/>
@@ -4249,12 +4253,12 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>Omalizumab:</t>
+          <t>Antagonistą receptora adenozynowego A2 jest:</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>jest przeciwciałem monoklonalnym anty-IgE</t>
+          <t>teofilina</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr"/>
@@ -4263,22 +4267,22 @@
       <c r="J73" s="2" t="inlineStr"/>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>hamuje fosfodiesterazę typu 2</t>
+          <t>meksyletyna</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>jest agonistą receptorów beta-2</t>
+          <t>sotalol</t>
         </is>
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>hamuje fosfolipazę A2</t>
+          <t>mianseryna</t>
         </is>
       </c>
       <c r="N73" s="2" t="inlineStr">
         <is>
-          <t>działa hamująco na receptory dla leukotrienów</t>
+          <t>finasteryd</t>
         </is>
       </c>
       <c r="O73" s="2" t="inlineStr"/>
@@ -4286,7 +4290,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>UKŁAD ODDECHOWY</t>
+          <t>LEKI PRZECIWDEPRESYJNE</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -4302,12 +4306,12 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Antagonistą receptora adenozynowego A2 jest:</t>
+          <t>Antagonistą receptora 5-HT2 jest:</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
-          <t>teofilina</t>
+          <t>trazodon</t>
         </is>
       </c>
       <c r="G74" s="2" t="inlineStr"/>
@@ -4316,22 +4320,22 @@
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr">
         <is>
-          <t>meksyletyna</t>
+          <t>mirtazapina</t>
         </is>
       </c>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>sotalol</t>
+          <t>moklobemid</t>
         </is>
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>mianseryna</t>
+          <t>dezypramina</t>
         </is>
       </c>
       <c r="N74" s="2" t="inlineStr">
         <is>
-          <t>finasteryd</t>
+          <t>wenlafaksyna</t>
         </is>
       </c>
       <c r="O74" s="2" t="inlineStr"/>
@@ -4344,7 +4348,7 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>Mechanizm działania</t>
+          <t>Wskazania</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr"/>
@@ -4355,12 +4359,12 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Antagonistą receptora 5-HT2 jest:</t>
+          <t>W leczeniu uzależnienia od nikotyny możesz zastosować:</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>trazodon</t>
+          <t>bupropion</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr"/>
@@ -4369,22 +4373,22 @@
       <c r="J75" s="2" t="inlineStr"/>
       <c r="K75" s="2" t="inlineStr">
         <is>
-          <t>mirtazapina</t>
+          <t>duloksetyna</t>
         </is>
       </c>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>moklobemid</t>
+          <t>ipsapiron</t>
         </is>
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>dezypramina</t>
+          <t>tropisetron</t>
         </is>
       </c>
       <c r="N75" s="2" t="inlineStr">
         <is>
-          <t>wenlafaksyna</t>
+          <t>zileuton</t>
         </is>
       </c>
       <c r="O75" s="2" t="inlineStr"/>
@@ -4392,12 +4396,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>LEKI PRZECIWDEPRESYJNE</t>
+          <t>NADCIŚNIENIE TĘTNICZE</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>Wskazania</t>
+          <t>Działania niepożądane</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr"/>
@@ -4408,12 +4412,12 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>W leczeniu uzależnienia od nikotyny możesz zastosować:</t>
+          <t>Silny kaszel może wystąpić podczas leczenia:</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>bupropion</t>
+          <t>chinapryl</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr"/>
@@ -4422,22 +4426,22 @@
       <c r="J76" s="2" t="inlineStr"/>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>duloksetyna</t>
+          <t>walsartan</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>ipsapiron</t>
+          <t>jodek potasu</t>
         </is>
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>tropisetron</t>
+          <t>minoksydyl</t>
         </is>
       </c>
       <c r="N76" s="2" t="inlineStr">
         <is>
-          <t>zileuton</t>
+          <t>eplerenon</t>
         </is>
       </c>
       <c r="O76" s="2" t="inlineStr"/>
@@ -4445,12 +4449,12 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>NADCIŚNIENIE TĘTNICZE</t>
+          <t>UKŁAD PRZYWSPÓŁCZULNY</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>Działania niepożądane</t>
+          <t>Wskazania</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr"/>
@@ -4461,12 +4465,12 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Silny kaszel może wystąpić podczas leczenia:</t>
+          <t>W celu rozszerzenia źrenicy celem diagnostyki zmian na dnie oka możesz zastosować:</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
-          <t>chinapryl</t>
+          <t>tropikamid</t>
         </is>
       </c>
       <c r="G77" s="2" t="inlineStr"/>
@@ -4475,22 +4479,22 @@
       <c r="J77" s="2" t="inlineStr"/>
       <c r="K77" s="2" t="inlineStr">
         <is>
-          <t>walsartan</t>
+          <t>pirazynamid</t>
         </is>
       </c>
       <c r="L77" s="2" t="inlineStr">
         <is>
-          <t>jodek potasu</t>
+          <t>topiramat</t>
         </is>
       </c>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>minoksydyl</t>
+          <t>pirydostygmina</t>
         </is>
       </c>
       <c r="N77" s="2" t="inlineStr">
         <is>
-          <t>eplerenon</t>
+          <t>donepezil</t>
         </is>
       </c>
       <c r="O77" s="2" t="inlineStr"/>
@@ -4498,12 +4502,12 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>UKŁAD PRZYWSPÓŁCZULNY</t>
+          <t>LEKI PRZECIWPSYCHOTYCZNE</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>Wskazania</t>
+          <t>Działania niepożądane</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr"/>
@@ -4514,12 +4518,12 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>W celu rozszerzenia źrenicy celem diagnostyki zmian na dnie oka możesz zastosować:</t>
+          <t>U pacjenta leczonego przez wiele lat z powodu schizofrenii występują działania niepożądane: akinezja, sztywność i drżenie. Są one wynikiem:</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
-          <t>tropikamid</t>
+          <t>działania przeciwdopaminergicznego</t>
         </is>
       </c>
       <c r="G78" s="2" t="inlineStr"/>
@@ -4528,22 +4532,22 @@
       <c r="J78" s="2" t="inlineStr"/>
       <c r="K78" s="2" t="inlineStr">
         <is>
-          <t>pirazynamid</t>
+          <t>działania przeciwcholinergicznego</t>
         </is>
       </c>
       <c r="L78" s="2" t="inlineStr">
         <is>
-          <t>topiramat</t>
+          <t>obniżenia ekspresji kwasu gamma-aminomasłowego (GABA)</t>
         </is>
       </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>pirydostygmina</t>
+          <t>hamowania wychwytu zwrotnego serotoniny</t>
         </is>
       </c>
       <c r="N78" s="2" t="inlineStr">
         <is>
-          <t>donepezil</t>
+          <t>działania przeciwserotoninowego</t>
         </is>
       </c>
       <c r="O78" s="2" t="inlineStr"/>
@@ -4551,7 +4555,7 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>LEKI PRZECIWPSYCHOTYCZNE</t>
+          <t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -4567,12 +4571,12 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>U pacjenta leczonego przez wiele lat z powodu schizofrenii występują działania niepożądane: akinezja, sztywność i drżenie. Są one wynikiem:</t>
+          <t>Pacjentka zostaje przyjęta do szpitala po spożyciu co najmniej 30 tabletek nieznanego leku. Wstępne badanie fizykalne nie wykazuje żadnych nieprawidłowości. Trzydzieści sześć godzin później aktywność ASPAT w surowicy wynosi 1500 U/L, a ALAT 2000 U/L. Jaki to lek?</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
-          <t>działania przeciwdopaminergicznego</t>
+          <t>paracetamol</t>
         </is>
       </c>
       <c r="G79" s="2" t="inlineStr"/>
@@ -4581,22 +4585,22 @@
       <c r="J79" s="2" t="inlineStr"/>
       <c r="K79" s="2" t="inlineStr">
         <is>
-          <t>działania przeciwcholinergicznego</t>
+          <t>kodeina</t>
         </is>
       </c>
       <c r="L79" s="2" t="inlineStr">
         <is>
-          <t>obniżenia ekspresji kwasu gamma-aminomasłowego (GABA)</t>
+          <t>ebastyna</t>
         </is>
       </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>hamowania wychwytu zwrotnego serotoniny</t>
+          <t>diazepam</t>
         </is>
       </c>
       <c r="N79" s="2" t="inlineStr">
         <is>
-          <t>działania przeciwserotoninowego</t>
+          <t>salbutamol</t>
         </is>
       </c>
       <c r="O79" s="2" t="inlineStr"/>
@@ -4604,12 +4608,12 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>NIEOPIOIDOWE LEKI PRZECIWBÓLOWE</t>
+          <t>UKŁAD POKARMOWY</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>Działania niepożądane</t>
+          <t>Mechanizm działania</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr"/>
@@ -4620,12 +4624,12 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Pacjentka zostaje przyjęta do szpitala po spożyciu co najmniej 30 tabletek nieznanego leku. Wstępne badanie fizykalne nie wykazuje żadnych nieprawidłowości. Trzydzieści sześć godzin później aktywność ASPAT w surowicy wynosi 1500 U/L, a ALAT 2000 U/L. Jaki to lek?</t>
+          <t>Omeprazol:</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
-          <t>paracetamol</t>
+          <t>hamuje aktywność H+/K+-ATPazy</t>
         </is>
       </c>
       <c r="G80" s="2" t="inlineStr"/>
@@ -4634,22 +4638,22 @@
       <c r="J80" s="2" t="inlineStr"/>
       <c r="K80" s="2" t="inlineStr">
         <is>
-          <t>kodeina</t>
+          <t>jest antagonistą receptorów dla gastryny</t>
         </is>
       </c>
       <c r="L80" s="2" t="inlineStr">
         <is>
-          <t>ebastyna</t>
+          <t>jest antagonistą receptorów H2</t>
         </is>
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>diazepam</t>
+          <t>jest antagonistą receptorów M3</t>
         </is>
       </c>
       <c r="N80" s="2" t="inlineStr">
         <is>
-          <t>salbutamol</t>
+          <t>jest analogiem prostaglandyny E</t>
         </is>
       </c>
       <c r="O80" s="2" t="inlineStr"/>
@@ -4657,12 +4661,12 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>UKŁAD POKARMOWY</t>
+          <t>LEKI PRZECIWBAKTERYJNE</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>Mechanizm działania</t>
+          <t>Interakcje</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr"/>
@@ -4673,12 +4677,12 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>Omeprazol:</t>
+          <t>Pacjentka przychodzi do lekarza z powodu nudności, wymiotów i bólów brzucha godzinę po spożyciu kieliszka wina do kolacji. Trzy dni temu zaczęła leczenie zakażenia rzęsistkiem pochwowym. Jaki lek przyjmuje pacjentka?</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>hamuje aktywność H+/K+-ATPazy</t>
+          <t>metronidazol</t>
         </is>
       </c>
       <c r="G81" s="2" t="inlineStr"/>
@@ -4687,22 +4691,22 @@
       <c r="J81" s="2" t="inlineStr"/>
       <c r="K81" s="2" t="inlineStr">
         <is>
-          <t>jest antagonistą receptorów dla gastryny</t>
+          <t>ceftriakson</t>
         </is>
       </c>
       <c r="L81" s="2" t="inlineStr">
         <is>
-          <t>jest antagonistą receptorów H2</t>
+          <t>chlorochina</t>
         </is>
       </c>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>jest antagonistą receptorów M3</t>
+          <t>doksycyklina</t>
         </is>
       </c>
       <c r="N81" s="2" t="inlineStr">
         <is>
-          <t>jest analogiem prostaglandyny E</t>
+          <t>mebendazol</t>
         </is>
       </c>
       <c r="O81" s="2" t="inlineStr"/>
@@ -4715,7 +4719,7 @@
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>Interakcje</t>
+          <t>Mechanizm działania</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr"/>
@@ -4726,12 +4730,12 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Pacjentka przychodzi do lekarza z powodu nudności, wymiotów i bólów brzucha godzinę po spożyciu kieliszka wina do kolacji. Trzy dni temu zaczęła leczenie zakażenia rzęsistkiem pochwowym. Jaki lek przyjmuje pacjentka?</t>
+          <t>U pacjenta z zakażeniem HIV i zapaleniem płuc wywołanym przez Pneumocystis jirovecii zastosowano skuteczne leczenie trimetoprimem-sulfametoksazolem dzięki hamowaniu aktywności:</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
-          <t>metronidazol</t>
+          <t>reduktazy dihydrofolianowej</t>
         </is>
       </c>
       <c r="G82" s="2" t="inlineStr"/>
@@ -4740,22 +4744,22 @@
       <c r="J82" s="2" t="inlineStr"/>
       <c r="K82" s="2" t="inlineStr">
         <is>
-          <t>ceftriakson</t>
+          <t>wbudowania steroli do błon komórkowych</t>
         </is>
       </c>
       <c r="L82" s="2" t="inlineStr">
         <is>
-          <t>chlorochina</t>
+          <t>kwasu p-aminobenzoesowego</t>
         </is>
       </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>doksycyklina</t>
+          <t>topoizomerazy II</t>
         </is>
       </c>
       <c r="N82" s="2" t="inlineStr">
         <is>
-          <t>mebendazol</t>
+          <t>syntezy białka PBP</t>
         </is>
       </c>
       <c r="O82" s="2" t="inlineStr"/>
@@ -4763,12 +4767,12 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>LEKI PRZECIWBAKTERYJNE</t>
+          <t>HEMOSTAZA</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>Mechanizm działania</t>
+          <t>Antidotum</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr"/>
@@ -4779,12 +4783,12 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>U pacjenta z zakażeniem HIV i zapaleniem płuc wywołanym przez Pneumocystis jirovecii zastosowano skuteczne leczenie trimetoprimem-sulfametoksazolem dzięki hamowaniu aktywności:</t>
+          <t>Odwrócenie efektu przeciwzakrzepowego heparyny uzyskasz po podaniu:</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>reduktazy dihydrofolianowej</t>
+          <t>siarczan protaminy</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr"/>
@@ -4793,22 +4797,22 @@
       <c r="J83" s="2" t="inlineStr"/>
       <c r="K83" s="2" t="inlineStr">
         <is>
-          <t>wbudowania steroli do błon komórkowych</t>
+          <t>heparynaza</t>
         </is>
       </c>
       <c r="L83" s="2" t="inlineStr">
         <is>
-          <t>kwasu p-aminobenzoesowego</t>
+          <t>kwas traneksamowy</t>
         </is>
       </c>
       <c r="M83" s="2" t="inlineStr">
         <is>
-          <t>topoizomerazy II</t>
+          <t>witamina K</t>
         </is>
       </c>
       <c r="N83" s="2" t="inlineStr">
         <is>
-          <t>syntezy białka PBP</t>
+          <t>antytrombina III</t>
         </is>
       </c>
       <c r="O83" s="2" t="inlineStr"/>
@@ -4816,12 +4820,12 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>HEMOSTAZA</t>
+          <t>LEKI PRZECIWDEPRESYJNE</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Antidotum</t>
+          <t>Działania niepożądane</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr"/>
@@ -4832,12 +4836,12 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Odwrócenie efektu przeciwzakrzepowego heparyny uzyskasz po podaniu:</t>
+          <t>Przedawkowanie trójpierścieniowych leków przeciwdepresyjnych może doprowadzić do zgonu pacjenta w wyniku:</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
-          <t>siarczan protaminy</t>
+          <t>zaburzeń rytmu serca</t>
         </is>
       </c>
       <c r="G84" s="2" t="inlineStr"/>
@@ -4846,22 +4850,22 @@
       <c r="J84" s="2" t="inlineStr"/>
       <c r="K84" s="2" t="inlineStr">
         <is>
-          <t>heparynaza</t>
+          <t>depresji ośrodka oddechowego</t>
         </is>
       </c>
       <c r="L84" s="2" t="inlineStr">
         <is>
-          <t>kwas traneksamowy</t>
+          <t>śpiączki</t>
         </is>
       </c>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>witamina K</t>
+          <t>hipertermii</t>
         </is>
       </c>
       <c r="N84" s="2" t="inlineStr">
         <is>
-          <t>antytrombina III</t>
+          <t>ostrej niewydolności nerek</t>
         </is>
       </c>
       <c r="O84" s="2" t="inlineStr"/>
@@ -4874,7 +4878,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Działania niepożądane</t>
+          <t>Mechanizm działania</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr"/>
@@ -4885,12 +4889,12 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Przedawkowanie trójpierścieniowych leków przeciwdepresyjnych może doprowadzić do zgonu pacjenta w wyniku:</t>
+          <t>Mechanizm działania litu w psychozie maniakalno-depresyjnej jest związany z:</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>zaburzeń rytmu serca</t>
+          <t>hamowaniem przemian fosfatydyloinozytoli w komórce</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr"/>
@@ -4899,22 +4903,22 @@
       <c r="J85" s="2" t="inlineStr"/>
       <c r="K85" s="2" t="inlineStr">
         <is>
-          <t>depresji ośrodka oddechowego</t>
+          <t>hamowaniem wychwytu zwrotnego noradrenaliny</t>
         </is>
       </c>
       <c r="L85" s="2" t="inlineStr">
         <is>
-          <t>śpiączki</t>
+          <t>hamowaniem wychwytu zwrotnego serotoniny</t>
         </is>
       </c>
       <c r="M85" s="2" t="inlineStr">
         <is>
-          <t>hipertermii</t>
+          <t>działaniem antagonistycznym na receptory dopaminergiczne D2</t>
         </is>
       </c>
       <c r="N85" s="2" t="inlineStr">
         <is>
-          <t>ostrej niewydolności nerek</t>
+          <t>działaniem cholinolitycznym</t>
         </is>
       </c>
       <c r="O85" s="2" t="inlineStr"/>
@@ -4922,12 +4926,12 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>LEKI PRZECIWDEPRESYJNE</t>
+          <t>FARMAKOKINETYKA</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Mechanizm działania</t>
+          <t>Farmakokinetyka</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr"/>
@@ -4938,12 +4942,12 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>Mechanizm działania litu w psychozie maniakalno-depresyjnej jest związany z:</t>
+          <t>Indeks terapeutyczny jest miarą:</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
-          <t>hamowaniem przemian fosfatydyloinozytoli w komórce</t>
+          <t>bezpieczeństwa</t>
         </is>
       </c>
       <c r="G86" s="2" t="inlineStr"/>
@@ -4952,22 +4956,22 @@
       <c r="J86" s="2" t="inlineStr"/>
       <c r="K86" s="2" t="inlineStr">
         <is>
-          <t>hamowaniem wychwytu zwrotnego noradrenaliny</t>
+          <t>siły działania leku</t>
         </is>
       </c>
       <c r="L86" s="2" t="inlineStr">
         <is>
-          <t>hamowaniem wychwytu zwrotnego serotoniny</t>
+          <t>selektywności</t>
         </is>
       </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>działaniem antagonistycznym na receptory dopaminergiczne D2</t>
+          <t>skuteczności</t>
         </is>
       </c>
       <c r="N86" s="2" t="inlineStr">
         <is>
-          <t>działaniem cholinolitycznym</t>
+          <t>stopnia wiązania z białkami krwi</t>
         </is>
       </c>
       <c r="O86" s="2" t="inlineStr"/>
@@ -4975,12 +4979,12 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>FARMAKOKINETYKA</t>
+          <t>ZNIECZULENIA OGÓLNE</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Farmakokinetyka</t>
+          <t>Działania niepożądane</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr"/>
@@ -4991,12 +4995,12 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>Indeks terapeutyczny jest miarą:</t>
+          <t>Z którym z następujących działań niepożądanych jest związane działanie ketaminy?</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
-          <t>bezpieczeństwa</t>
+          <t>omamy i koszmary senne</t>
         </is>
       </c>
       <c r="G87" s="2" t="inlineStr"/>
@@ -5005,22 +5009,22 @@
       <c r="J87" s="2" t="inlineStr"/>
       <c r="K87" s="2" t="inlineStr">
         <is>
-          <t>siły działania leku</t>
+          <t>podrażnienie dróg oddechowych</t>
         </is>
       </c>
       <c r="L87" s="2" t="inlineStr">
         <is>
-          <t>selektywności</t>
+          <t>obniżenie objętości wyrzutowej serca</t>
         </is>
       </c>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>skuteczności</t>
+          <t>hipertermia złośliwa</t>
         </is>
       </c>
       <c r="N87" s="2" t="inlineStr">
         <is>
-          <t>stopnia wiązania z białkami krwi</t>
+          <t>rabdomioliza</t>
         </is>
       </c>
       <c r="O87" s="2" t="inlineStr"/>
@@ -5028,12 +5032,12 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>ZNIECZULENIA OGÓLNE</t>
+          <t>UKŁAD PRZYWSPÓŁCZULNY</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Działania niepożądane</t>
+          <t>Antidotum</t>
         </is>
       </c>
       <c r="C88" s="2" t="inlineStr"/>
@@ -5044,12 +5048,12 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>Z którym z następujących działań niepożądanych jest związane działanie ketaminy?</t>
+          <t>Pacjent z łzawieniem, wymiotami i biegunką, puls 45/min, ciśnienie tętnicze 90/60 mm Hg. Objawy mogą wskazywać na zatrucie:</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>omamy i koszmary senne</t>
+          <t>związkami fosforoorganicznymi</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr"/>
@@ -5058,22 +5062,22 @@
       <c r="J88" s="2" t="inlineStr"/>
       <c r="K88" s="2" t="inlineStr">
         <is>
-          <t>podrażnienie dróg oddechowych</t>
+          <t>metanolem</t>
         </is>
       </c>
       <c r="L88" s="2" t="inlineStr">
         <is>
-          <t>obniżenie objętości wyrzutowej serca</t>
+          <t>toksyną botulinową</t>
         </is>
       </c>
       <c r="M88" s="2" t="inlineStr">
         <is>
-          <t>hipertermia złośliwa</t>
+          <t>glikolem etylenowym</t>
         </is>
       </c>
       <c r="N88" s="2" t="inlineStr">
         <is>
-          <t>rabdomioliza</t>
+          <t>digoksyną</t>
         </is>
       </c>
       <c r="O88" s="2" t="inlineStr"/>
@@ -5081,12 +5085,12 @@
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>UKŁAD PRZYWSPÓŁCZULNY</t>
+          <t>LEKI PRZECIWGRZYBICZE</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>Antidotum</t>
+          <t>Wskazania</t>
         </is>
       </c>
       <c r="C89" s="2" t="inlineStr"/>
@@ -5097,12 +5101,12 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>Pacjent z łzawieniem, wymiotami i biegunką, puls 45/min, ciśnienie tętnicze 90/60 mm Hg. Objawy mogą wskazywać na zatrucie:</t>
+          <t>U pacjentki leczonej z powodu ostrej białaczki limfoblastycznej stwierdzono powikłanie – obecność Candida albicans w surowicy. Który z poniższych leków przeciwgrzybiczych należy zastosować?</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>związkami fosforoorganicznymi</t>
+          <t>amfoterycyna B</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr"/>
@@ -5111,22 +5115,22 @@
       <c r="J89" s="2" t="inlineStr"/>
       <c r="K89" s="2" t="inlineStr">
         <is>
-          <t>metanolem</t>
+          <t>nystatyna</t>
         </is>
       </c>
       <c r="L89" s="2" t="inlineStr">
         <is>
-          <t>toksyną botulinową</t>
+          <t>klotrimazol</t>
         </is>
       </c>
       <c r="M89" s="2" t="inlineStr">
         <is>
-          <t>glikolem etylenowym</t>
+          <t>ketokonazol</t>
         </is>
       </c>
       <c r="N89" s="2" t="inlineStr">
         <is>
-          <t>digoksyną</t>
+          <t>kapsaicyna</t>
         </is>
       </c>
       <c r="O89" s="2" t="inlineStr"/>
@@ -5150,12 +5154,12 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>U pacjentki leczonej z powodu ostrej białaczki limfoblastycznej stwierdzono powikłanie – obecność Candida albicans w surowicy. Który z poniższych leków przeciwgrzybiczych należy zastosować?</t>
+          <t>U pacjenta z AIDS rozwija się gorączka, ból szyi i światłowstręt. Badanie płynu mózgowo-rdzeniowego ujawnia Cryptococcus neoformans. Który z leków zastosować?</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>amfoterycyna B</t>
+          <t>flukonazol</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr"/>
@@ -5164,22 +5168,22 @@
       <c r="J90" s="2" t="inlineStr"/>
       <c r="K90" s="2" t="inlineStr">
         <is>
-          <t>nystatyna</t>
+          <t>flucytozyna</t>
         </is>
       </c>
       <c r="L90" s="2" t="inlineStr">
         <is>
-          <t>klotrimazol</t>
+          <t>gryzeofulwina</t>
         </is>
       </c>
       <c r="M90" s="2" t="inlineStr">
         <is>
-          <t>ketokonazol</t>
+          <t>cykloseryna</t>
         </is>
       </c>
       <c r="N90" s="2" t="inlineStr">
         <is>
-          <t>kapsaicyna</t>
+          <t>kotrimoksazol</t>
         </is>
       </c>
       <c r="O90" s="2" t="inlineStr"/>
@@ -5187,7 +5191,7 @@
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>LEKI PRZECIWGRZYBICZE</t>
+          <t>LEKI PRZECIWPASOŻYTNICZE</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -5203,12 +5207,12 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>U pacjenta z AIDS rozwija się gorączka, ból szyi i światłowstręt. Badanie płynu mózgowo-rdzeniowego ujawnia Cryptococcus neoformans. Który z leków zastosować?</t>
+          <t>Jaki lek przeciwmalaryczny należy zastosować profilaktycznie w przypadku podróży do rejonu z opornością na chlorochinę?</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
-          <t>flukonazol</t>
+          <t>meflochina</t>
         </is>
       </c>
       <c r="G91" s="2" t="inlineStr"/>
@@ -5217,22 +5221,22 @@
       <c r="J91" s="2" t="inlineStr"/>
       <c r="K91" s="2" t="inlineStr">
         <is>
-          <t>flucytozyna</t>
+          <t>prymachina</t>
         </is>
       </c>
       <c r="L91" s="2" t="inlineStr">
         <is>
-          <t>gryzeofulwina</t>
+          <t>doksycyklina</t>
         </is>
       </c>
       <c r="M91" s="2" t="inlineStr">
         <is>
-          <t>cykloseryna</t>
+          <t>pirymetamina</t>
         </is>
       </c>
       <c r="N91" s="2" t="inlineStr">
         <is>
-          <t>kotrimoksazol</t>
+          <t>ryfampicyna</t>
         </is>
       </c>
       <c r="O91" s="2" t="inlineStr"/>
@@ -5256,12 +5260,12 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Jaki lek przeciwmalaryczny należy zastosować profilaktycznie w przypadku podróży do rejonu z opornością na chlorochinę?</t>
+          <t>W zakażeniu Giardia lamblia możesz zastosować:</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
-          <t>meflochina</t>
+          <t>metronidazol</t>
         </is>
       </c>
       <c r="G92" s="2" t="inlineStr"/>
@@ -5270,22 +5274,22 @@
       <c r="J92" s="2" t="inlineStr"/>
       <c r="K92" s="2" t="inlineStr">
         <is>
-          <t>prymachina</t>
+          <t>nifurtimoks</t>
         </is>
       </c>
       <c r="L92" s="2" t="inlineStr">
         <is>
-          <t>doksycyklina</t>
+          <t>mebendazol</t>
         </is>
       </c>
       <c r="M92" s="2" t="inlineStr">
         <is>
-          <t>pirymetamina</t>
+          <t>suramina</t>
         </is>
       </c>
       <c r="N92" s="2" t="inlineStr">
         <is>
-          <t>ryfampicyna</t>
+          <t>pyrantel</t>
         </is>
       </c>
       <c r="O92" s="2" t="inlineStr"/>
@@ -5309,12 +5313,12 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>W zakażeniu Giardia lamblia możesz zastosować:</t>
+          <t>W leczeniu zakażenia Toxoplasma gondii jest stosowana:</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>metronidazol</t>
+          <t>pirymetamina</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr"/>
@@ -5323,22 +5327,22 @@
       <c r="J93" s="2" t="inlineStr"/>
       <c r="K93" s="2" t="inlineStr">
         <is>
-          <t>nifurtimoks</t>
+          <t>iwermektyna</t>
         </is>
       </c>
       <c r="L93" s="2" t="inlineStr">
         <is>
-          <t>mebendazol</t>
+          <t>prazykwantel</t>
         </is>
       </c>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>suramina</t>
+          <t>niklozamid</t>
         </is>
       </c>
       <c r="N93" s="2" t="inlineStr">
         <is>
-          <t>pyrantel</t>
+          <t>tiabendazol</t>
         </is>
       </c>
       <c r="O93" s="2" t="inlineStr"/>
@@ -5346,7 +5350,7 @@
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>LEKI PRZECIWPASOŻYTNICZE</t>
+          <t>UKŁAD POKARMOWY</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
@@ -5362,12 +5366,12 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>W leczeniu zakażenia Toxoplasma gondii jest stosowana:</t>
+          <t>Pacjent z podwyższonym stężeniem w surowicy wazoaktywnego peptydu jelitowego w związku z nowotworem trzustki (VIP-oma) powinien otrzymać:</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>pirymetamina</t>
+          <t>oktreotyd</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr"/>
@@ -5376,22 +5380,22 @@
       <c r="J94" s="2" t="inlineStr"/>
       <c r="K94" s="2" t="inlineStr">
         <is>
-          <t>iwermektyna</t>
+          <t>gastryna</t>
         </is>
       </c>
       <c r="L94" s="2" t="inlineStr">
         <is>
-          <t>prazykwantel</t>
+          <t>glukagon</t>
         </is>
       </c>
       <c r="M94" s="2" t="inlineStr">
         <is>
-          <t>niklozamid</t>
+          <t>sulfasalazyna</t>
         </is>
       </c>
       <c r="N94" s="2" t="inlineStr">
         <is>
-          <t>tiabendazol</t>
+          <t>famotydyna</t>
         </is>
       </c>
       <c r="O94" s="2" t="inlineStr"/>
@@ -5415,12 +5419,12 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Pacjent z podwyższonym stężeniem w surowicy wazoaktywnego peptydu jelitowego w związku z nowotworem trzustki (VIP-oma) powinien otrzymać:</t>
+          <t>U pacjenta z rozpoznaniem zespołu Zollingera-Ellisona możesz zastosować:</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
-          <t>oktreotyd</t>
+          <t>lansoprazol</t>
         </is>
       </c>
       <c r="G95" s="2" t="inlineStr"/>
@@ -5429,22 +5433,22 @@
       <c r="J95" s="2" t="inlineStr"/>
       <c r="K95" s="2" t="inlineStr">
         <is>
-          <t>gastryna</t>
+          <t>famotydyna</t>
         </is>
       </c>
       <c r="L95" s="2" t="inlineStr">
         <is>
-          <t>glukagon</t>
+          <t>mizoprostol</t>
         </is>
       </c>
       <c r="M95" s="2" t="inlineStr">
         <is>
-          <t>sulfasalazyna</t>
+          <t>propantelina</t>
         </is>
       </c>
       <c r="N95" s="2" t="inlineStr">
         <is>
-          <t>famotydyna</t>
+          <t>cytrynian potasowo-bizmutawy</t>
         </is>
       </c>
       <c r="O95" s="2" t="inlineStr"/>
@@ -5452,7 +5456,7 @@
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>UKŁAD POKARMOWY</t>
+          <t>NADCIŚNIENIE TĘTNICZE</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
@@ -5468,12 +5472,12 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>U pacjenta z rozpoznaniem zespołu Zollingera-Ellisona możesz zastosować:</t>
+          <t>U pacjenta z nadciśnieniem tętniczym i współistniejącym białkomoczem celowe jest zastosowanie:</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>lansoprazol</t>
+          <t>peryndopryl</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr"/>
@@ -5482,22 +5486,22 @@
       <c r="J96" s="2" t="inlineStr"/>
       <c r="K96" s="2" t="inlineStr">
         <is>
-          <t>famotydyna</t>
+          <t>nikardypina</t>
         </is>
       </c>
       <c r="L96" s="2" t="inlineStr">
         <is>
-          <t>mizoprostol</t>
+          <t>nitrogliceryna</t>
         </is>
       </c>
       <c r="M96" s="2" t="inlineStr">
         <is>
-          <t>propantelina</t>
+          <t>hydrochlorotiazyd</t>
         </is>
       </c>
       <c r="N96" s="2" t="inlineStr">
         <is>
-          <t>cytrynian potasowo-bizmutawy</t>
+          <t>moksonidyna</t>
         </is>
       </c>
       <c r="O96" s="2" t="inlineStr"/>
@@ -5505,12 +5509,12 @@
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>NADCIŚNIENIE TĘTNICZE</t>
+          <t>PADACZKA</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>Wskazania</t>
+          <t>Działania niepożądane</t>
         </is>
       </c>
       <c r="C97" s="2" t="inlineStr"/>
@@ -5521,12 +5525,12 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>U pacjenta z nadciśnieniem tętniczym i współistniejącym białkomoczem celowe jest zastosowanie:</t>
+          <t>Hepatotoksyczne działanie wykazuje:</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>peryndopryl</t>
+          <t>kwas walproinowy</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr"/>
@@ -5535,22 +5539,22 @@
       <c r="J97" s="2" t="inlineStr"/>
       <c r="K97" s="2" t="inlineStr">
         <is>
-          <t>nikardypina</t>
+          <t>cetyryzyna</t>
         </is>
       </c>
       <c r="L97" s="2" t="inlineStr">
         <is>
-          <t>nitrogliceryna</t>
+          <t>mupirocyna</t>
         </is>
       </c>
       <c r="M97" s="2" t="inlineStr">
         <is>
-          <t>hydrochlorotiazyd</t>
+          <t>penicylina krystaliczna</t>
         </is>
       </c>
       <c r="N97" s="2" t="inlineStr">
         <is>
-          <t>moksonidyna</t>
+          <t>bromheksyna</t>
         </is>
       </c>
       <c r="O97" s="2" t="inlineStr"/>
@@ -5558,12 +5562,12 @@
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>PADACZKA</t>
+          <t>STANY NAGŁE</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Działania niepożądane</t>
+          <t>Wskazania</t>
         </is>
       </c>
       <c r="C98" s="2" t="inlineStr"/>
@@ -5574,12 +5578,12 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>Hepatotoksyczne działanie wykazuje:</t>
+          <t>U 60-letniego chorego z obrzękiem płuc i ciśnieniem krwi 190/110 mmHg zastosujesz:</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>kwas walproinowy</t>
+          <t>nitrogliceryna we wlewie dożylnym</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr"/>
@@ -5588,22 +5592,22 @@
       <c r="J98" s="2" t="inlineStr"/>
       <c r="K98" s="2" t="inlineStr">
         <is>
-          <t>cetyryzyna</t>
+          <t>nifedypina podjęzykowo</t>
         </is>
       </c>
       <c r="L98" s="2" t="inlineStr">
         <is>
-          <t>mupirocyna</t>
+          <t>kaptopryl doustnie</t>
         </is>
       </c>
       <c r="M98" s="2" t="inlineStr">
         <is>
-          <t>penicylina krystaliczna</t>
+          <t>klonidyna doustnie</t>
         </is>
       </c>
       <c r="N98" s="2" t="inlineStr">
         <is>
-          <t>bromheksyna</t>
+          <t>amiodaron dożylnie</t>
         </is>
       </c>
       <c r="O98" s="2" t="inlineStr"/>
@@ -5611,12 +5615,12 @@
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>STANY NAGŁE</t>
+          <t>UKŁAD WSPÓŁCZULNY</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Wskazania</t>
+          <t>Działania niepożądane</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr"/>
@@ -5627,12 +5631,12 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>U 60-letniego chorego z obrzękiem płuc i ciśnieniem krwi 190/110 mmHg zastosujesz:</t>
+          <t>Ksylometazolina:</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>nitrogliceryna we wlewie dożylnym</t>
+          <t>może doprowadzić do wystąpienia tzw. „efektu z odbicia”</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr"/>
@@ -5641,81 +5645,28 @@
       <c r="J99" s="2" t="inlineStr"/>
       <c r="K99" s="2" t="inlineStr">
         <is>
-          <t>nifedypina podjęzykowo</t>
+          <t>jest antagonistą receptorów alfa</t>
         </is>
       </c>
       <c r="L99" s="2" t="inlineStr">
         <is>
-          <t>kaptopryl doustnie</t>
+          <t>skuteczność kliniczną wykazuje po 5 dniach terapii</t>
         </is>
       </c>
       <c r="M99" s="2" t="inlineStr">
         <is>
-          <t>klonidyna doustnie</t>
+          <t>jest podawana doustnie</t>
         </is>
       </c>
       <c r="N99" s="2" t="inlineStr">
         <is>
-          <t>amiodaron dożylnie</t>
+          <t>dobrze penetruje przez barierę krew-mózg</t>
         </is>
       </c>
       <c r="O99" s="2" t="inlineStr"/>
     </row>
-    <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>UKŁAD WSPÓŁCZULNY</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>Działania niepożądane</t>
-        </is>
-      </c>
-      <c r="C100" s="2" t="inlineStr"/>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>testowe</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>Ksylometazolina:</t>
-        </is>
-      </c>
-      <c r="F100" s="2" t="inlineStr">
-        <is>
-          <t>może doprowadzić do wystąpienia tzw. „efektu z odbicia”</t>
-        </is>
-      </c>
-      <c r="G100" s="2" t="inlineStr"/>
-      <c r="H100" s="2" t="inlineStr"/>
-      <c r="I100" s="2" t="inlineStr"/>
-      <c r="J100" s="2" t="inlineStr"/>
-      <c r="K100" s="2" t="inlineStr">
-        <is>
-          <t>jest antagonistą receptorów alfa</t>
-        </is>
-      </c>
-      <c r="L100" s="2" t="inlineStr">
-        <is>
-          <t>skuteczność kliniczną wykazuje po 5 dniach terapii</t>
-        </is>
-      </c>
-      <c r="M100" s="2" t="inlineStr">
-        <is>
-          <t>jest podawana doustnie</t>
-        </is>
-      </c>
-      <c r="N100" s="2" t="inlineStr">
-        <is>
-          <t>dobrze penetruje przez barierę krew-mózg</t>
-        </is>
-      </c>
-      <c r="O100" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:O100"/>
+  <autoFilter ref="A1:O99"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>